<commit_message>
Build site at 2021-05-18 15:02:08 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Publicacoes/eleno.xlsx
+++ b/_Drive/Publicacoes/eleno.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>DOI</t>
   </si>
@@ -115,13 +115,16 @@
   </si>
   <si>
     <t>10.1088/1361-6668/abf7cf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.jallcom.2021.160411</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -136,6 +139,10 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -156,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -165,6 +172,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -550,7 +560,11 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" ht="12.75" customHeight="1"/>
+    <row r="34" ht="12.75" customHeight="1">
+      <c r="A34" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
     <row r="35" ht="12.75" customHeight="1"/>
     <row r="36" ht="12.75" customHeight="1"/>
     <row r="37" ht="12.75" customHeight="1"/>
@@ -1520,6 +1534,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="A33"/>
+    <hyperlink r:id="rId2" ref="A34"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.6666666666666667" footer="0.0" header="0.0" left="1.0" right="1.0" top="1.6666666666666667"/>
@@ -1528,6 +1543,6 @@
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-05-18 15:07:12 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Publicacoes/eleno.xlsx
+++ b/_Drive/Publicacoes/eleno.xlsx
@@ -117,14 +117,14 @@
     <t>10.1088/1361-6668/abf7cf</t>
   </si>
   <si>
-    <t>https://doi.org/10.1016/j.jallcom.2021.160411</t>
+    <t>10.1016/j.jallcom.2021.160411</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -141,11 +141,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-    </font>
-    <font>
-      <u/>
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
@@ -163,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -172,9 +167,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -561,7 +553,7 @@
       </c>
     </row>
     <row r="34" ht="12.75" customHeight="1">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1532,10 +1524,6 @@
     <row r="999" ht="12.75" customHeight="1"/>
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="A33"/>
-    <hyperlink r:id="rId2" ref="A34"/>
-  </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.6666666666666667" footer="0.0" header="0.0" left="1.0" right="1.0" top="1.6666666666666667"/>
   <pageSetup paperSize="9" cellComments="atEnd" orientation="portrait"/>
@@ -1543,6 +1531,6 @@
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>